<commit_message>
Cap nhat Danh-muc-24-tam_A-313-3.xlsx theo trang thai moi nhat (2026-10-24)
- Y3: anh ro (chup lai a252-254), dau hoi 213->155, NE PROSLEZHENO 166->95.
- Y4: tu CHUA CO -> da chep PARTIAL dang ke (BOM 80, net 794 chan, kiem
  cheo 133 khop/25 lech ten/1 chi-E3/3 chi-E4, con ~207 NE PROSLEZHENO +
  C3-C8 chua lan).
- Y5: soat lai bang anh ro, dau hoi 169->84, chi-E4 36->35, 3 lech ten
  da chot cach doc.
- Y6, Y16: cap nhat duong dan anh theo ten moi (khong doi so lieu noi dung).
- Doi 'Chua ro - cho chup lai' -> 'Ro' (mau xanh) cho ca 5 tam tren.
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -67,7 +67,7 @@
       <sz val="9"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +104,12 @@
         <fgColor rgb="FFF2F2F2"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6E0B4"/>
+        <bgColor rgb="FFC6E0B4"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -132,7 +138,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -166,6 +172,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -549,7 +558,7 @@
       <c r="A1" s="12" t="inlineStr">
         <is>
           <t>DANH MỤC 24 TẤM A-313-3 — SỐ HIỆU &amp; TÌNH TRẠNG SƠ ĐỒ Э3 (ảnh chụp bản giấy ЕУ3.048.002 РЭ)
-Nguồn: SO-DO-DAU-NOI_E4_A-313-3.md §2 (danh mục cấp khối tr.142, đã chốt) + DANH-MUC_ANH_RE_A-313-3.md §2  |  Cập nhật: 2026-10-23</t>
+Nguồn: SO-DO-DAU-NOI_E4_A-313-3.md §2 (danh mục cấp khối tr.142, đã chốt) + DANH-MUC_ANH_RE_A-313-3.md §2  |  Cập nhật: 2026-10-24</t>
         </is>
       </c>
     </row>
@@ -688,17 +697,17 @@
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t>158–161 (#155–#158) + tờ 1 chụp lại #231/#232</t>
-        </is>
-      </c>
-      <c r="F6" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>158–161 (#155–#158) + tờ 1 (A313-3_CONTROL/Y3/RE_trXXX_a252.jpg, RE_tr160_a253.jpg, RE_tr161_a254.jpg, chụp lại rõ 2026-10-24)</t>
+        </is>
+      </c>
+      <c r="F6" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>Claude chép: BOM 99, 818 chân, 166 chân НЕ ПРОСЛЕЖЕНО, 213 dòng '?'. Cần chụp lại rõ tờ 2/3; chưa rõ #155/#156 có thuộc hình này không.</t>
+          <t>Claude chép: BOM 99, 818 chân. SAU chụp lại rõ 2026-10-24 (phiên khác): dấu hỏi giảm 213→155, НЕ ПРОСЛЕЖЕНО giảm 166→95. e3_vs_e4.py 6 У3: 125 khớp/32 lệch tên (phần lớn cách ghi →↔⇒, 3п↔Зп)/1 chỉ-Э3/9 chỉ-Э4. Chi tiết ric06_mota.md.</t>
         </is>
       </c>
     </row>
@@ -720,22 +729,22 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>CHƯA CÓ</t>
+          <t>Có một phần (PARTIAL, đã chép đáng kể, 2026-10-24)</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>— (chưa thấy trang nào)</t>
-        </is>
-      </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>158–159 (#155, #156), chụp lại rõ A313-3_CONTROL/Y4/RE_tr158_a250.jpg (tờ 1/2), RE_tr159_a251.jpg (tờ 2/2)</t>
+        </is>
+      </c>
+      <c r="F7" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
         <is>
-          <t>Hoàn toàn chưa chụp được sơ đồ nguyên lý. Chỉ có ПЭ #137–#139 (trang chưa đọc được).</t>
+          <t>Chụp lại rõ 2026-10-24, chép qua Codex (prompt do Claude soát/sửa — bổ sung R11 thiếu trong đề bài gốc). BOM 80 ref (R1-R12 trừ R9/R10 gạch bỏ, C1-C8, 61 vi mạch; KHÔNG có У8/У22/У24/У27 trong ПЭ, khớp đúng chỗ gạch trên Э3). Net 794 chân (2 tờ). e3_vs_e4.py 5 У4 (176 hàng П1/П2/П3): 133 khớp/25 lệch tên (phần lớn cách ghi)/1 chỉ-Э3/3 chỉ-Э4. Còn: ~207 chân НЕ ПРОСЛЕЖЕНО (chủ yếu thanh dọc bộ giải mã tờ 1) + C3-C8 chưa lần chân (ngoại lệ đã biết, tụ lọc nguồn). Chưa xác định chắc a251 là trang 159 hay 189. Chi tiết ric05_mota.md.</t>
         </is>
       </c>
     </row>
@@ -757,22 +766,22 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Có một phần (PARTIAL, đã chép)</t>
+          <t>Có một phần (PARTIAL, soát lại 2026-10-24, giảm đáng kể)</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>171–172 (#167, #168)</t>
-        </is>
-      </c>
-      <c r="F8" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>171–172, chụp lại rõ A313-3_CONTROL/Y5/RE_tr171_a263.jpg, RE_tr172_a264.jpg (thay bản mờ #167/#168 cũ)</t>
+        </is>
+      </c>
+      <c r="F8" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>T03b: 169 dòng '?' còn, 36 chân chỉ-Э4 chưa soát. Ảnh #168 cần chụp lại rõ hơn.</t>
+          <t>T03/T03b (ảnh cũ mờ): 86 ref, 948 chân, 169 '?', 36 chỉ-Э4. SAU chụp lại rõ + soát lại 2026-10-24 (87 lượt vision_analyze qua subagent, Claude kiểm lại và sửa 2 lỗi quy ước trước khi nhận): '?' giảm 169→84 (~50%), chỉ-Э4 giảm 36→35, cả 3 lệch tên đã chốt cách đọc (П2/2='R15' viết đè; П3/42 xác nhận thật khác Э4; П1/10='Вход.П ТТЛ'). e3_vs_e4.py 8 У5: 125 chân Э3, khớp 122, chỉ-Э4 35. Còn 84 '?' với lý do cụ thể: У9/У10/У17/У18 bus dọc chồng khít không tách điểm nối; У24 + một phần У25 không tìm thấy vị trí vật lý trên ảnh; vài chân У20/У22/У23 có thể không dùng. Chi tiết PROJECT_HANDOFF.md T06b.</t>
         </is>
       </c>
     </row>
@@ -799,12 +808,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>164–166 (#161–#163); trang 167 thiếu</t>
-        </is>
-      </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>164–166, chụp lại rõ A313-3_CONTROL/Y6/RE_trXXX_a255.jpg…a257.jpg (л.1-3/3)</t>
+        </is>
+      </c>
+      <c r="F9" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1169,7 +1178,7 @@
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>tr.153-157 (л.1-5, A313-3_CONTROL/Y16/E3_matran_lis1-5_*.jpg, 2 bộ ảnh/lист)</t>
+          <t>tr.153-157 (л.1-5): RE_tr153_a150.jpg…RE_tr157_a154.jpg (chụp gốc) + RE_trXXX_a258.jpg…a262.jpg (chụp lại rõ 2026-10-24), A313-3_CONTROL/Y16/</t>
         </is>
       </c>
       <c r="F19" s="4" t="inlineStr">

</xml_diff>

<commit_message>
A-313-3: Excel danh muc dong Y6 cap nhat; PROJECT_HANDOFF §13-14 (Y3/Y4/Y6)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -803,7 +803,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>ĐÃ CHÉP PARTIAL (Codex chép, Claude kiểm): ric07_bom.csv 77 dòng, ric07_net.csv 997 chân, ric07_conn.csv 173 chân (П1/П2/П3). ric07_vs_e4.csv: 139 chân Э3/157 chân Э4, khớp 103, lệch tên 36, chỉ-Э4 18.</t>
+          <t>ĐÃ CHÉP PARTIAL (Codex chép, Codex soát lại, Claude áp + kiểm): ric07_bom.csv 77 dòng, ric07_net.csv 997 chân (còn 175 dòng "?"), ric07_conn.csv 173 chân. ric07_vs_e4.csv: khớp 105, lệch tên 38, chỉ-Э4 14.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -818,7 +818,7 @@
       </c>
       <c r="G9" s="6" t="inlineStr">
         <is>
-          <t>3 tờ nhưng thiếu tờ ứng với trang 167. Chưa đưa vào hàng đợi chép (T0x). | Ảnh thay 2026-10-24: 3 ảnh cũ mờ (tr.164-166) -&gt; 3 ảnh chụp lại rõ (л.1-3/3), xác nhận mã ЕУ3.057.140. Chép Э3 2026-10-24 (Codex qua Hermes): toàn bộ tên linh kiện BOM ghi "?"; 184/997 dòng net "?". Kiểm chéo Э3↔Э4: khớp 103/139, 36 lệch tên phần lớn do viết tắt khác nhau (không phải lỗi thật), 1 nghi đọc nhầm ТТП/ТТЛ tại П2/2-5. Chi tiết: PROJECT_HANDOFF.md T06.</t>
+          <t>3 tờ nhưng thiếu tờ ứng với trang 167. Chưa đưa vào hàng đợi chép (T0x). | Ảnh thay 2026-10-24: 3 ảnh cũ mờ (tr.164-166) -&gt; 3 ảnh chụp lại rõ (л.1-3/3), xác nhận mã ЕУ3.057.140. Chép Э3 2026-10-24 (Codex qua Hermes): toàn bộ tên linh kiện BOM ghi "?"; 184/997 dòng net "?". Kiểm chéo Э3↔Э4: khớp 103/139, 36 lệch tên phần lớn do viết tắt khác nhau (không phải lỗi thật), 1 nghi đọc nhầm ТТП/ТТЛ tại П2/2-5. Chi tiết: PROJECT_HANDOFF.md T06. | Soát lại 2026-10-24: 23/196 dòng "?" đọc chắc (ric07_soat_raw.csv, ric07_soat_apply.py); 4 ô bảng mới đọc khớp Э4. Chưa vào e3_check (14 ref "?", 4 pin "?"). Chưa có ПЭ рис.7 → 77 linh kiện chưa có trị số. Nên chụp lại л.2/л.3 độ phân giải cao hơn.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Y11: thay anh ro net du ca to, xoa anh cu, bat dau giao chep
- 2 anh moi xac nhan dung Y11 (EU2.242.113 E3, l.1/2 tr202, l.2/2 tr203) -
  chup lai du ca to (anh cu chi chup 1 phan theo ghi chu truoc).
- Xoa RE_tr202_a204.jpg, RE_tr203_a205.jpg (mo/thieu), doi ten anh moi
  RE_tr202_a266.jpg, RE_tr203_a267.jpg theo quy tac.
- Anh thu 3 (bo mach that, khong phai so do giay) doi ten
  anh-bo-mach-that_2026-10-24.jpg, khong theo quy tac RE_tr_a (quy tac do
  chi danh cho anh chup ban giay).
- Cap nhat DANH-MUC_ANH_RE_A-313-3.md (dong Y11, so a cao nhat a267),
  Danh-muc-24-tam_A-313-3.xlsx (dong Y11: Ro, dang chep).
- Giao subagent chep moi ric17 (BOM tu PE tr204-205 + netlist tu 2 anh
  so do) - dang chay nen.
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -993,17 +993,17 @@
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>202–203 (#204, #205)</t>
-        </is>
-      </c>
-      <c r="F14" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>202–203, chụp lại rõ nét đủ cả tờ 2026-10-24: A313-3_CONTROL/Y11/RE_tr202_a266.jpg (л.1/2), RE_tr203_a267.jpg (л.2/2)</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G14" s="3" t="inlineStr">
         <is>
-          <t>Tờ gấp chỉ chụp 1 phần (theo DANH-MUC §4). Có thay thế tạm ✅ A313-V.05.</t>
+          <t>Ảnh cũ chỉ chụp 1 phần tờ gấp — đã thay bằng 2 ảnh chụp lại đủ cả tờ (л.1/2, л.2/2), mã ЕУ2.242.113 Э3 xác nhận rõ. Có thêm ảnh bo mạch thật (anh-bo-mach-that_2026-10-24.jpg) để đối chiếu. Đang giao subagent chép BOM (từ ПЭ tr.204-205) + netlist — xem PROJECT_HANDOFF.md khi hoàn tất.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel danh muc: dong Y10 da chep (ric.18)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -969,7 +969,7 @@
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>Có ảnh, chưa chép</t>
+          <t>ĐÃ CHÉP (Claude, 2026-10-25): ric18_bom.csv 82 ref, ric18_net.csv 425 chân, ric18_conn.csv П1 53 chân; e3_check PASS; Э3↔Э4 39 khớp / 4 lệch tên / 1 chỉ-Э4.</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -984,7 +984,7 @@
       </c>
       <c r="G13" s="6" t="inlineStr">
         <is>
-          <t>Có thay thế tạm ◐ A313-V.06 (cùng chức năng, khác mạch).</t>
+          <t>Có thay thế tạm ◐ A313-V.06 (cùng chức năng, khác mạch). | 2026-10-25: chép từ RE_tr206_a208 (nét hơn ảnh chụp lại). Cùng topo A313-V.06; М/~М = «УПР МОД.1/2» theo Э4; đế 168КТ2 nối +6,3/+3,5 В (khác .06). Chi tiết ric18_mota.md.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
A-313-3 Y1: cap nhat Excel danh muc (dong Y1) sau khi nguoi dung dong file
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -636,7 +636,7 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Có — ảnh đã rõ (chưa chép Э3↔Э4)</t>
+          <t>Có một phần (PARTIAL, chép lần đầu 2026-10-25)</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr">
@@ -646,12 +646,12 @@
       </c>
       <c r="F4" s="4" t="inlineStr">
         <is>
-          <t>Rõ</t>
+          <t>Rõ (chép ric10_*)</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>Chụp lại rõ nét 2026-10-23: đọc được đầy đủ ký hiệu linh kiện (У65, У64, У41, У51...), số chân, nhãn tín hiệu (П3/28(1), Тпр, ВходПК1 13-16разр...), bảng А/Б 0-15. Chưa thấy khung tên (số рис/mã ký hiệu) trong vùng đã chụp — có thể ở tờ khác. Còn thiếu: đối chiếu #75 (tr.79/80) có thuộc hình này không; chưa chép BOM/net.</t>
+          <t>Chép PARTIAL 2026-10-25: dataset ric10_* trong tmp/pdfs/review/a313-3/e3/. Nguồn 2 tờ: RE_tr179_a175.jpg (tờ 1, tr.179) + RE_trXXX_a075.jpg (tờ 2, kẹp tr.79/80, 'tờ #75'). Ảnh Y1.jpg (PCB thật, upload GitHub) không dùng làm nguồn chép. BOM 82 ref; net 115 dòng (53 truy trực tiếp, 62 placeholder — lý do khối lượng linh kiện, không phải hỏng ảnh cụ thể); bảng П3 48 dòng (designator đọc trực tiếp, xác nhận qua spot-check) + 2 bảng phụ П3-right-1/2 chưa rõ designator (mép phải trang bị cắt khi chụp). check_ric10.py PASS (coordinator chạy lại độc lập khớp). Coordinator sửa 1 lỗi nhỏ của subagent (designator П3 thực có in, không phải suy luận). CHƯA xác nhận 100% tờ 1 và tờ 2 có cùng một bản vẽ — xem ric10_mota.md. 2 trùng ref giữ minh bạch: У44/У44b, R29/R29b.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel danh muc: cap nhat trang thai Y17 va Y21 (ca hai da chep xong, PASS, anh ro)
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -1244,7 +1244,7 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>BOM+net+tính toán 25% tải. Lắp ráp Рис.33(?) tr.247 — khung tên CHƯA đọc được (xem dòng riêng bên dưới), suy luận theo chuỗi số. CHỤP LẠI RÕ 2026-10-25: RE_tr231_a269.jpg thay ảnh cũ #233 (mờ/gập góc, đã xoá). Soát lại ric25_*: xác nhận Д3/Д4 THỰC SỰ không vẽ trên trang này (có trong перечень, không có trên Э3); sửa hướng mũi tên T24 (NPN); xác nhận R16/R17, Д23, nhóm Д34…Д40 (1 ký hiệu dùng nhãn khoảng). netlist vẫn 397 dòng/164 BOM, 5 dòng ? còn lại (node шина M, vấn đề hiểu mạch không phải ảnh mờ). Coordinator spot-check độc lập khớp.</t>
+          <t>BOM 164 ref, net 397 dòng (164 BOM/397 net khớp chéo, 0 chân trùng, 0 net mồ côi). CHỤP LẠI RÕ 2026-10-25: RE_tr231_a269.jpg thay ảnh cũ #233 (mờ/gập góc, đã xoá). Soát lại ric25_*: xác nhận Д3/Д4 THỰC SỰ không vẽ trên trang này (có trong перечень, không có trên Э3); sửa hướng mũi tên T24 (NPN); xác nhận R16/R17, Д23, nhóm Д34…Д40 (1 ký hiệu dùng nhãn khoảng). Còn 5 dòng "?" (node шина M, vấn đề hiểu mạch không phải ảnh mờ — cần đo trên tấm thật). Coordinator spot-check độc lập khớp (Д3/Д4 vắng mặt, hướng T24).</t>
         </is>
       </c>
     </row>
@@ -1402,22 +1402,22 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Có, đã chép nhưng còn thiếu ảnh phụ</t>
+          <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
         <is>
-          <t>221 (#221); ПЭ #222 + tr.222 thiếu</t>
+          <t>221 (#221, đã thay bằng a270 2026-10-25); ПЭ #222-224 (trong archive gốc, không phải ảnh working riêng)</t>
         </is>
       </c>
       <c r="F25" s="7" t="inlineStr">
         <is>
-          <t>Chưa rõ — chờ chụp lại</t>
+          <t>Rõ</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
         <is>
-          <t>Mâu thuẫn trị số điện áp: kế hoạch ghi −23V theo Bảng 3, nhưng Э4 có cả hai (У16КП1/5 ghi '−23В', 3Ш3В/60 ghi '−20В'). Thiếu ảnh ПЭ tr.222.</t>
+          <t>BOM 44 ref, net 100 dòng; checker e3_ric2223.py: bom∖net=[], net∖bom=[], chân trùng=[], net &lt;2 chân=[] — SẠCH. CHỤP LẠI RÕ 2026-10-25: RE_tr221_a270.jpg thay ảnh cũ #221 (mờ). ĐÃ XÁC NHẬN chấm nối lá 7 ↔ C5…C8/anode Д2 (N13) — trước đây nghi ngờ do ảnh mờ không thấy chấm nối, nay thấy rõ. Xác nhận nhãn Д2, R16. Mâu thuẫn trị số vẫn còn, KHÔNG phải do ảnh: Пр1 ghi "1А" trên Э3 vs перечень "2А" — cần xem nhãn trên tấm thật; biến thể −02 (−23 В; 0,25 А) theo HDSD/Э4 chưa có Э3/перечень riêng (chỉ có bản gốc −20 В); mức logic X:1 (chân điều khiển) chưa rõ nguồn ngoài kéo lên mức nào.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Excel Danh-muc-24-tam: xoa dong Y17-lap rap (ban ve bo tri chi tham khao), them ghi chu vao Y17 va LUU Y
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
+++ b/Excel center control/Danh-muc-24-tam_A-313-3.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="-285" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Danh muc 24 tam A-313-3" sheetId="1" state="visible" r:id="rId1"/>
@@ -194,14 +194,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -570,28 +570,28 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G38"/>
+  <dimension ref="A1:G39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="14" customWidth="1" style="14" min="1" max="1"/>
-    <col width="36" customWidth="1" style="14" min="2" max="2"/>
-    <col width="22" customWidth="1" style="14" min="3" max="3"/>
-    <col width="23" customWidth="1" style="14" min="4" max="4"/>
-    <col width="34" customWidth="1" style="14" min="5" max="5"/>
-    <col width="16" customWidth="1" style="14" min="6" max="6"/>
-    <col width="70" customWidth="1" style="14" min="7" max="7"/>
+    <col width="14" customWidth="1" style="15" min="1" max="1"/>
+    <col width="36" customWidth="1" style="15" min="2" max="2"/>
+    <col width="22" customWidth="1" style="15" min="3" max="3"/>
+    <col width="23" customWidth="1" style="15" min="4" max="4"/>
+    <col width="34" customWidth="1" style="15" min="5" max="5"/>
+    <col width="16" customWidth="1" style="15" min="6" max="6"/>
+    <col width="70" customWidth="1" style="15" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="34" customHeight="1" s="14">
-      <c r="A1" s="15" t="inlineStr">
+    <row r="1" ht="34" customHeight="1" s="15">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>DANH MỤC 24 TẤM A-313-3 — SỐ HIỆU &amp; TÌNH TRẠNG SƠ ĐỒ Э3 (ảnh chụp bản giấy ЕУ3.048.002 РЭ)
-Nguồn: SO-DO-DAU-NOI_E4_A-313-3.md §2 (danh mục cấp khối tr.142, đã chốt) + DANH-MUC_ANH_RE_A-313-3.md §2  |  Cập nhật: 2026-10-25</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="14" customHeight="1" s="14"/>
-    <row r="3" ht="24" customHeight="1" s="14">
+Nguồn: SO-DO-DAU-NOI_E4_A-313-3.md §2 (danh mục cấp khối tr.142, đã chốt) + DANH-MUC_ANH_RE_A-313-3.md §2  |  Cập nhật: 2026-10-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="14" customHeight="1" s="15"/>
+    <row r="3" ht="24" customHeight="1" s="15">
       <c r="A3" s="1" t="inlineStr">
         <is>
           <t>Vị trí</t>
@@ -628,7 +628,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="58" customHeight="1" s="14">
+    <row r="4" ht="58" customHeight="1" s="15">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Y1</t>
@@ -665,7 +665,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1" s="14">
+    <row r="5" ht="58" customHeight="1" s="15">
       <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Y2</t>
@@ -702,7 +702,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="58" customHeight="1" s="14">
+    <row r="6" ht="58" customHeight="1" s="15">
       <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Y3</t>
@@ -739,7 +739,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="58" customHeight="1" s="14">
+    <row r="7" ht="58" customHeight="1" s="15">
       <c r="A7" s="5" t="inlineStr">
         <is>
           <t>Y4</t>
@@ -776,7 +776,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="58" customHeight="1" s="14">
+    <row r="8" ht="58" customHeight="1" s="15">
       <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Y5</t>
@@ -813,7 +813,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="58" customHeight="1" s="14">
+    <row r="9" ht="58" customHeight="1" s="15">
       <c r="A9" s="5" t="inlineStr">
         <is>
           <t>Y6</t>
@@ -850,7 +850,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="58" customHeight="1" s="14">
+    <row r="10" ht="58" customHeight="1" s="15">
       <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Y7</t>
@@ -887,7 +887,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="58" customHeight="1" s="14">
+    <row r="11" ht="58" customHeight="1" s="15">
       <c r="A11" s="5" t="inlineStr">
         <is>
           <t>Y8</t>
@@ -924,7 +924,7 @@
         </is>
       </c>
     </row>
-    <row r="12" ht="58" customHeight="1" s="14">
+    <row r="12" ht="58" customHeight="1" s="15">
       <c r="A12" s="2" t="inlineStr">
         <is>
           <t>Y9</t>
@@ -961,7 +961,7 @@
         </is>
       </c>
     </row>
-    <row r="13" ht="58" customHeight="1" s="14">
+    <row r="13" ht="58" customHeight="1" s="15">
       <c r="A13" s="5" t="inlineStr">
         <is>
           <t>Y10</t>
@@ -998,7 +998,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="58" customHeight="1" s="14">
+    <row r="14" ht="58" customHeight="1" s="15">
       <c r="A14" s="2" t="inlineStr">
         <is>
           <t>Y11</t>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="58" customHeight="1" s="14">
+    <row r="15" ht="58" customHeight="1" s="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
           <t>Y12</t>
@@ -1072,7 +1072,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="58" customHeight="1" s="14">
+    <row r="16" ht="58" customHeight="1" s="15">
       <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Y13</t>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="58" customHeight="1" s="14">
+    <row r="17" ht="58" customHeight="1" s="15">
       <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Y14</t>
@@ -1146,7 +1146,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="58" customHeight="1" s="14">
+    <row r="18" ht="58" customHeight="1" s="15">
       <c r="A18" s="2" t="inlineStr">
         <is>
           <t>Y15</t>
@@ -1183,7 +1183,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="58" customHeight="1" s="14">
+    <row r="19" ht="58" customHeight="1" s="15">
       <c r="A19" s="5" t="inlineStr">
         <is>
           <t>Y16</t>
@@ -1220,7 +1220,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="58" customHeight="1" s="14">
+    <row r="20" ht="58" customHeight="1" s="15">
       <c r="A20" s="2" t="inlineStr">
         <is>
           <t>Y17</t>
@@ -1253,104 +1253,100 @@
       </c>
       <c r="G20" s="3" t="inlineStr">
         <is>
-          <t>BOM 164 ref, net 397 dòng (164 BOM/397 net khớp chéo, 0 chân trùng, 0 net mồ côi). CHỤP LẠI RÕ 2026-10-25: RE_tr231_a269.jpg thay ảnh cũ #233 (mờ/gập góc, đã xoá). Soát lại ric25_*: xác nhận Д3/Д4 THỰC SỰ không vẽ trên trang này (có trong перечень, không có trên Э3); sửa hướng mũi tên T24 (NPN); xác nhận R16/R17, Д23, nhóm Д34…Д40 (1 ký hiệu dùng nhãn khoảng). Còn 5 dòng "?" (node шина M, vấn đề hiểu mạch không phải ảnh mờ — cần đo trên tấm thật). Coordinator spot-check độc lập khớp (Д3/Д4 vắng mặt, hướng T24).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="58" customHeight="1" s="14">
-      <c r="A21" s="5" t="inlineStr">
-        <is>
-          <t>Y17-lắp ráp</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>УЛП 5В 15А — bản vẽ lắp ráp (Д7)</t>
-        </is>
-      </c>
-      <c r="C21" s="5" t="inlineStr">
-        <is>
-          <t>ВШ6.730.530 (nghi, theo KE-HOACH)</t>
-        </is>
-      </c>
-      <c r="D21" s="5" t="inlineStr">
-        <is>
-          <t>Có ảnh, khung tên chưa đọc được</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>247 (#248); nghi thiếu tiếp tr.248+ (рис.34?)</t>
-        </is>
-      </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>Chưa rõ — chờ chụp lại</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>KE-HOACH tiên đoán Рис.33/34 = ВШ6.730.527/530 Д7 — khớp suy luận theo chuỗi 27→28→29→30→31→32→33. Khung tên thật nằm ngoài vùng ảnh đã chụp. ⚠ CẦN CHỤP LẠI để xác nhận.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="58" customHeight="1" s="14">
-      <c r="A22" s="2" t="inlineStr">
+          <t>BOM 164 ref, net 397 dòng (164 BOM/397 net khớp chéo, 0 chân trùng, 0 net mồ côi). CHỤP LẠI RÕ 2026-10-25: RE_tr231_a269.jpg thay ảnh cũ #233 (mờ/gập góc, đã xoá). Soát lại ric25_*: xác nhận Д3/Д4 THỰC SỰ không vẽ trên trang này (có trong перечень, không có trên Э3); sửa hướng mũi tên T24 (NPN); xác nhận R16/R17, Д23, nhóm Д34…Д40 (1 ký hiệu dùng nhãn khoảng). Còn 5 dòng "?" (node шина M, vấn đề hiểu mạch không phải ảnh mờ — cần đo trên tấm thật). Coordinator spot-check độc lập khớp (Д3/Д4 vắng mặt, hướng T24). | Ảnh bố trí tr.247–248 (ВШ6.730.530 Д7, *_bo-tri.jpg) CHỈ để tham khảo vị trí linh kiện trên tấm thật, không phải sơ đồ — không nằm trong danh mục (người dùng, 2026-10-26).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="58" customHeight="1" s="15">
+      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Y18</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>УЛП +20 В 0,3 А</t>
         </is>
       </c>
-      <c r="C22" s="2" t="inlineStr">
+      <c r="C21" s="2" t="inlineStr">
         <is>
           <t>ЕУ3.215.446</t>
         </is>
       </c>
-      <c r="D22" s="2" t="inlineStr">
+      <c r="D21" s="2" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E21" s="3" t="inlineStr">
         <is>
           <t>214 (#215)</t>
         </is>
       </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t>Rõ</t>
+        </is>
+      </c>
+      <c r="G21" s="3" t="n"/>
+    </row>
+    <row r="22" ht="58" customHeight="1" s="15">
+      <c r="A22" s="5" t="inlineStr">
+        <is>
+          <t>Y19</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>УЛП +12,6 В 1 А</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>ЕУ3.215.452</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Có — đã chép xong (PASS)</t>
+        </is>
+      </c>
+      <c r="E22" s="6" t="inlineStr">
+        <is>
+          <t>225 (#225)</t>
+        </is>
+      </c>
       <c r="F22" s="4" t="inlineStr">
         <is>
           <t>Rõ</t>
         </is>
       </c>
-      <c r="G22" s="3" t="n"/>
-    </row>
-    <row r="23" ht="58" customHeight="1" s="14">
-      <c r="A23" s="5" t="inlineStr">
-        <is>
-          <t>Y19</t>
-        </is>
-      </c>
-      <c r="B23" s="6" t="inlineStr">
-        <is>
-          <t>УЛП +12,6 В 1 А</t>
-        </is>
-      </c>
-      <c r="C23" s="5" t="inlineStr">
-        <is>
-          <t>ЕУ3.215.452</t>
-        </is>
-      </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="G22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="58" customHeight="1" s="15">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Y20</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>УЛП +6,3 В 0,5 А</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>ЕУ3.215.448-01</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E23" s="6" t="inlineStr">
-        <is>
-          <t>225 (#225)</t>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>218 (#219)</t>
         </is>
       </c>
       <c r="F23" s="4" t="inlineStr">
@@ -1358,102 +1354,106 @@
           <t>Rõ</t>
         </is>
       </c>
-      <c r="G23" s="6" t="n"/>
-    </row>
-    <row r="24" ht="58" customHeight="1" s="14">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Y20</t>
-        </is>
-      </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>УЛП +6,3 В 0,5 А</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="inlineStr">
-        <is>
-          <t>ЕУ3.215.448-01</t>
-        </is>
-      </c>
-      <c r="D24" s="2" t="inlineStr">
+      <c r="G23" s="3" t="n"/>
+    </row>
+    <row r="24" ht="58" customHeight="1" s="15">
+      <c r="A24" s="5" t="inlineStr">
+        <is>
+          <t>Y21</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t>УЛП −20 В (hoặc −23 В — mâu thuẫn trị số) 0,25–0,3 А</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>ЕУ3.215.451</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
-        <is>
-          <t>218 (#219)</t>
-        </is>
-      </c>
-      <c r="F24" s="4" t="inlineStr">
-        <is>
-          <t>Rõ</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="n"/>
-    </row>
-    <row r="25" ht="58" customHeight="1" s="14">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>Y21</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t>УЛП −20 В (hoặc −23 В — mâu thuẫn trị số) 0,25–0,3 А</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t>ЕУ3.215.451</t>
-        </is>
-      </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="E24" s="6" t="inlineStr">
+        <is>
+          <t>221 (#221, đã thay bằng a270 2026-10-25); ПЭ #222-224 (trong archive gốc, không phải ảnh working riêng)</t>
+        </is>
+      </c>
+      <c r="F24" s="13" t="inlineStr">
+        <is>
+          <t>Rõ</t>
+        </is>
+      </c>
+      <c r="G24" s="6" t="inlineStr">
+        <is>
+          <t>BOM 44 ref, net 100 dòng; checker e3_ric2223.py: bom∖net=[], net∖bom=[], chân trùng=[], net &lt;2 chân=[] — SẠCH. CHỤP LẠI RÕ 2026-10-25: RE_tr221_a270.jpg thay ảnh cũ #221 (mờ). ĐÃ XÁC NHẬN chấm nối lá 7 ↔ C5…C8/anode Д2 (N13) — trước đây nghi ngờ do ảnh mờ không thấy chấm nối, nay thấy rõ. Xác nhận nhãn Д2, R16. Mâu thuẫn trị số vẫn còn, KHÔNG phải do ảnh: Пр1 ghi "1А" trên Э3 vs перечень "2А" — cần xem nhãn trên tấm thật; biến thể −02 (−23 В; 0,25 А) theo HDSD/Э4 chưa có Э3/перечень riêng (chỉ có bản gốc −20 В); mức logic X:1 (chân điều khiển) chưa rõ nguồn ngoài kéo lên mức nào.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="58" customHeight="1" s="15">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>Y22</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>УЛП −12,6 В 1 А</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>ЕУ3.215.470</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E25" s="6" t="inlineStr">
-        <is>
-          <t>221 (#221, đã thay bằng a270 2026-10-25); ПЭ #222-224 (trong archive gốc, không phải ảnh working riêng)</t>
-        </is>
-      </c>
-      <c r="F25" s="16" t="inlineStr">
-        <is>
-          <t>Rõ</t>
-        </is>
-      </c>
-      <c r="G25" s="6" t="inlineStr">
-        <is>
-          <t>BOM 44 ref, net 100 dòng; checker e3_ric2223.py: bom∖net=[], net∖bom=[], chân trùng=[], net &lt;2 chân=[] — SẠCH. CHỤP LẠI RÕ 2026-10-25: RE_tr221_a270.jpg thay ảnh cũ #221 (mờ). ĐÃ XÁC NHẬN chấm nối lá 7 ↔ C5…C8/anode Д2 (N13) — trước đây nghi ngờ do ảnh mờ không thấy chấm nối, nay thấy rõ. Xác nhận nhãn Д2, R16. Mâu thuẫn trị số vẫn còn, KHÔNG phải do ảnh: Пр1 ghi "1А" trên Э3 vs перечень "2А" — cần xem nhãn trên tấm thật; biến thể −02 (−23 В; 0,25 А) theo HDSD/Э4 chưa có Э3/перечень riêng (chỉ có bản gốc −20 В); mức logic X:1 (chân điều khiển) chưa rõ nguồn ngoài kéo lên mức nào.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="58" customHeight="1" s="14">
-      <c r="A26" s="2" t="inlineStr">
-        <is>
-          <t>Y22</t>
-        </is>
-      </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>УЛП −12,6 В 1 А</t>
-        </is>
-      </c>
-      <c r="C26" s="2" t="inlineStr">
-        <is>
-          <t>ЕУ3.215.470</t>
-        </is>
-      </c>
-      <c r="D26" s="2" t="inlineStr">
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>237 (#239); ПЭ tr.238 thiếu</t>
+        </is>
+      </c>
+      <c r="F25" s="4" t="inlineStr">
+        <is>
+          <t>Rõ</t>
+        </is>
+      </c>
+      <c r="G25" s="3" t="inlineStr">
+        <is>
+          <t>Sơ đồ chính đã chép xong; chỉ thiếu 1 trang phụ lục ПЭ (238).</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="58" customHeight="1" s="15">
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Y23</t>
+        </is>
+      </c>
+      <c r="B26" s="6" t="inlineStr">
+        <is>
+          <t>УЛП ±10 В 0,2 А</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>ЕУ3.215.466</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
-        <is>
-          <t>237 (#239); ПЭ tr.238 thiếu</t>
+      <c r="E26" s="6" t="inlineStr">
+        <is>
+          <t>228 (#228)</t>
         </is>
       </c>
       <c r="F26" s="4" t="inlineStr">
@@ -1461,36 +1461,32 @@
           <t>Rõ</t>
         </is>
       </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Sơ đồ chính đã chép xong; chỉ thiếu 1 trang phụ lục ПЭ (238).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="58" customHeight="1" s="14">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>Y23</t>
-        </is>
-      </c>
-      <c r="B27" s="6" t="inlineStr">
-        <is>
-          <t>УЛП ±10 В 0,2 А</t>
-        </is>
-      </c>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>ЕУ3.215.466</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="G26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="58" customHeight="1" s="15">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>Y24</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Плата контроля и сигнализации</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>ЕУ2.072.139</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
         <is>
           <t>Có — đã chép xong (PASS)</t>
         </is>
       </c>
-      <c r="E27" s="6" t="inlineStr">
-        <is>
-          <t>228 (#228)</t>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>209 (#211)</t>
         </is>
       </c>
       <c r="F27" s="4" t="inlineStr">
@@ -1498,69 +1494,39 @@
           <t>Rõ</t>
         </is>
       </c>
-      <c r="G27" s="6" t="n"/>
-    </row>
-    <row r="28" ht="58" customHeight="1" s="14">
-      <c r="A28" s="2" t="inlineStr">
-        <is>
-          <t>Y24</t>
-        </is>
-      </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>Плата контроля и сигнализации</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="inlineStr">
-        <is>
-          <t>ЕУ2.072.139</t>
-        </is>
-      </c>
-      <c r="D28" s="2" t="inlineStr">
-        <is>
-          <t>Có — đã chép xong (PASS)</t>
-        </is>
-      </c>
-      <c r="E28" s="3" t="inlineStr">
-        <is>
-          <t>209 (#211)</t>
-        </is>
-      </c>
-      <c r="F28" s="4" t="inlineStr">
-        <is>
-          <t>Rõ</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Lắp ráp Рис.30 (tr.244) đã đọc rõ, khớp đúng mã ЕУ2.072.139 (khác Bảng 7 ghi ЕУ3.215.139).</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="28" s="15"/>
+    <row r="29" s="15">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>LƯU Ý:
   • Cột 'Số hiệu' lấy theo danh mục cấp khối tr.142 đã chốt (SO-DO-DAU-NOI_E4 §2) — là bản sửa so với KE-HOACH ban đầu (У12/У13 đảo, У21 = −20V không phải −23V, У24 = ЕУ2.072.139).
   • Y14/Y15: MÂU THUẪN chưa giải — ngay trong chính Э4 (tr.142 vs tr.149) đã ghi ngược nhau. Không dùng mã này để đặt hàng/đấu dây khi chưa đọc nhãn trên tấm thật.
   • Màu CAM ở cột 'Ảnh đã rõ chưa' = cần chụp lại (tờ gấp cắt mép, mất khung tên, hoặc chưa xác định được trang). Màu XANH = ảnh đủ rõ để dùng hoặc đã chép xong và kiểm chéo Э3↔Э4.
-  • Hàng 'Y17-lắp ráp' tách riêng khỏi Y17 vì đó là bản vẽ LẮP RÁP (Д7, khác sơ đồ nguyên lý Э3) — khung tên thật chưa chụp được, chỉ suy luận theo chuỗi số Рис. liên tục (27→33).
+  • Bản vẽ BỐ TRÍ/lắp ráp (Рис.27–34, tr.241–248, kể cả ВШ6.730.530 Д7 của Y17) KHÔNG phải sơ đồ để dùng, chỉ tham khảo vị trí khi xem tấm thật — không có dòng riêng trong danh mục này (đã bỏ dòng 'Y17-lắp ráp' 2026-10-26).
   • Nguồn &amp; phần nguyên lý còn thiếu: Y4 (hoàn toàn chưa có), Y9 (chưa xác định trang), Y16 (ưu tiên 1, chỉ có Э4).</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32"/>
-    <row r="33"/>
-    <row r="34"/>
-    <row r="35"/>
-    <row r="36"/>
-    <row r="37"/>
-    <row r="38"/>
+    <row r="30" s="15"/>
+    <row r="31" s="15"/>
+    <row r="32" s="15"/>
+    <row r="33" s="15"/>
+    <row r="34" s="15"/>
+    <row r="35" s="15"/>
+    <row r="36" s="15"/>
+    <row r="37" s="15"/>
+    <row r="38" s="15"/>
+    <row r="39" s="15"/>
   </sheetData>
   <autoFilter ref="A3:G3"/>
   <mergeCells count="2">
-    <mergeCell ref="A30:G38"/>
+    <mergeCell ref="A29:G37"/>
     <mergeCell ref="A1:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>